<commit_message>
more runs for the with_dn model
</commit_message>
<xml_diff>
--- a/model_code_book.xlsx
+++ b/model_code_book.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\1confiProj\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CFE368C-B2CC-4DAC-BDEE-80F6A2281E31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13958721-8873-427A-9AF1-7380492B1663}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9060" yWindow="1656" windowWidth="16668" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -88,12 +88,6 @@
 xdiff - Non-Bayesian measurement difference based estimation</t>
   </si>
   <si>
-    <t>0 - no decision noise
-1 - same decision noise for causal decision and confidence
-2 - only add decision noise for confidence but no causal decision
--1 - different decision noise for causal decision and confidence</t>
-  </si>
-  <si>
     <t>Decision noise indicator for Bayesian causal read-out</t>
   </si>
   <si>
@@ -157,6 +151,13 @@
     <t>0 - one shared parameter
 1 - two parameters
 2 - a fixed number</t>
+  </si>
+  <si>
+    <t>0 - no decision noise
+1 - same decision noise for causal decision and confidence
+2 - only add decision noise for confidence but no causal decision
+-1 - different decision noise for causal decision and confidence
+-2 - only add decision noise for causal decision but not confidence</t>
   </si>
 </sst>
 </file>
@@ -558,15 +559,15 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" ht="72" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>7</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
@@ -582,68 +583,68 @@
     </row>
     <row r="8" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="C8" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="C9" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="C10" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" t="s">
         <v>28</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B13" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
clean the analysis folder
</commit_message>
<xml_diff>
--- a/model_code_book.xlsx
+++ b/model_code_book.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\1confiProj\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13958721-8873-427A-9AF1-7380492B1663}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C964CBA-D4AB-4D4E-99BE-4E6110720029}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="40">
   <si>
     <t>FieldName</t>
   </si>
@@ -158,6 +158,16 @@
 2 - only add decision noise for confidence but no causal decision
 -1 - different decision noise for causal decision and confidence
 -2 - only add decision noise for causal decision but not confidence</t>
+  </si>
+  <si>
+    <t>linear_reduce</t>
+  </si>
+  <si>
+    <t>linear transformation or logistice transformation of the posterior prob of C to form a confidence</t>
+  </si>
+  <si>
+    <t>0-logistics
+1-linear</t>
   </si>
 </sst>
 </file>
@@ -222,8 +232,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{370B6285-FEF0-4A9B-85B6-14A2C6EFFA07}" name="Table1" displayName="Table1" ref="A1:C13" totalsRowShown="0">
-  <autoFilter ref="A1:C13" xr:uid="{370B6285-FEF0-4A9B-85B6-14A2C6EFFA07}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{370B6285-FEF0-4A9B-85B6-14A2C6EFFA07}" name="Table1" displayName="Table1" ref="A1:C14" totalsRowShown="0">
+  <autoFilter ref="A1:C14" xr:uid="{370B6285-FEF0-4A9B-85B6-14A2C6EFFA07}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{BF429E0C-3389-476D-ABCD-F23B1D39E634}" name="FieldName"/>
     <tableColumn id="3" xr3:uid="{08202248-299D-45A0-8B32-56E3AC87EDDC}" name="Description"/>
@@ -496,7 +506,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.33203125" bestFit="1" customWidth="1"/>
@@ -647,6 +657,17 @@
         <v>34</v>
       </c>
     </row>
+    <row r="14" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>37</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>